<commit_message>
five updated + readme
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -625,6 +625,66 @@
       </c>
       <c r="C13" t="n">
         <v>1115</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SDA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Usuario SDA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>QER</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Usuario QER</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>QWDQ</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Usuario QWDQ</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DQWD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Usuario DQWD</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>20000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>